<commit_message>
toiling. broke out means for policy and deservingness. fixing chapter 1.
</commit_message>
<xml_diff>
--- a/state_policy_eligibility.xlsx
+++ b/state_policy_eligibility.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kom11/Documents/GitHub/phd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD799DE-71B1-054D-8C40-8CBA772FA0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA49B8DD-5627-F446-85E3-6220665FB1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6640" yWindow="680" windowWidth="27560" windowHeight="19140" xr2:uid="{0358933F-5589-C549-9C92-1EC025553EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="171">
   <si>
     <t>State</t>
   </si>
@@ -715,19 +715,28 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -739,17 +748,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1085,7 +1085,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{254DB367-4C7D-D140-880A-139DA66ED8B7}">
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:M118"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="29" customWidth="1"/>
@@ -1093,7 +1093,7 @@
     <col min="5" max="5" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="69" thickBot="1">
+    <row r="1" spans="1:13" ht="69" thickBot="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1123,8 +1123,11 @@
       <c r="K1" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="17" thickBot="1">
+      <c r="M1" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="17" thickBot="1">
       <c r="A2" t="s">
         <v>168</v>
       </c>
@@ -1132,50 +1135,50 @@
         <v>170</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="34">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:13" ht="34">
+      <c r="A3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="19" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="15" t="s">
+      <c r="F3" s="19"/>
+      <c r="G3" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="19" t="s">
         <v>12</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="35" thickBot="1">
-      <c r="A4" s="16"/>
-      <c r="B4" s="17"/>
+    <row r="4" spans="1:13" ht="35" thickBot="1">
+      <c r="A4" s="26"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
       <c r="K4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18" thickBot="1">
-      <c r="A5" s="17"/>
+    <row r="5" spans="1:13" ht="18" thickBot="1">
+      <c r="A5" s="20"/>
       <c r="B5" s="7" t="s">
         <v>15</v>
       </c>
@@ -1197,8 +1200,8 @@
       </c>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" ht="171" thickBot="1">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:13" ht="188" thickBot="1">
+      <c r="A6" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -1226,8 +1229,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="35" thickBot="1">
-      <c r="A7" s="17"/>
+    <row r="7" spans="1:13" ht="35" thickBot="1">
+      <c r="A7" s="20"/>
       <c r="B7" s="7" t="s">
         <v>15</v>
       </c>
@@ -1251,8 +1254,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="205" thickBot="1">
-      <c r="A8" s="15" t="s">
+    <row r="8" spans="1:13" ht="239" thickBot="1">
+      <c r="A8" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="8" t="s">
@@ -1276,12 +1279,12 @@
       <c r="J8" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K8" s="15" t="s">
+      <c r="K8" s="19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="389" thickBot="1">
-      <c r="A9" s="17"/>
+    <row r="9" spans="1:13" ht="405" thickBot="1">
+      <c r="A9" s="20"/>
       <c r="B9" s="7" t="s">
         <v>15</v>
       </c>
@@ -1303,10 +1306,10 @@
       <c r="J9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K9" s="17"/>
-    </row>
-    <row r="10" spans="1:11" ht="52" thickBot="1">
-      <c r="A10" s="15" t="s">
+      <c r="K9" s="20"/>
+    </row>
+    <row r="10" spans="1:13" ht="69" thickBot="1">
+      <c r="A10" s="19" t="s">
         <v>25</v>
       </c>
       <c r="B10" s="8" t="s">
@@ -1334,8 +1337,8 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="120" thickBot="1">
-      <c r="A11" s="17"/>
+    <row r="11" spans="1:13" ht="120" thickBot="1">
+      <c r="A11" s="20"/>
       <c r="B11" s="7" t="s">
         <v>15</v>
       </c>
@@ -1361,8 +1364,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="137" thickBot="1">
-      <c r="A12" s="15" t="s">
+    <row r="12" spans="1:13" ht="137" thickBot="1">
+      <c r="A12" s="19" t="s">
         <v>31</v>
       </c>
       <c r="B12" s="8" t="s">
@@ -1386,12 +1389,12 @@
       <c r="J12" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K12" s="15" t="s">
+      <c r="K12" s="19" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="18" thickBot="1">
-      <c r="A13" s="17"/>
+    <row r="13" spans="1:13" ht="18" thickBot="1">
+      <c r="A13" s="20"/>
       <c r="B13" s="7" t="s">
         <v>34</v>
       </c>
@@ -1411,10 +1414,10 @@
       <c r="J13" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K13" s="17"/>
-    </row>
-    <row r="14" spans="1:11" ht="137" thickBot="1">
-      <c r="A14" s="15" t="s">
+      <c r="K13" s="20"/>
+    </row>
+    <row r="14" spans="1:13" ht="154" thickBot="1">
+      <c r="A14" s="19" t="s">
         <v>35</v>
       </c>
       <c r="B14" s="8" t="s">
@@ -1438,12 +1441,12 @@
       <c r="J14" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K14" s="15" t="s">
+      <c r="K14" s="19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="52" thickBot="1">
-      <c r="A15" s="17"/>
+    <row r="15" spans="1:13" ht="52" thickBot="1">
+      <c r="A15" s="20"/>
       <c r="B15" s="7" t="s">
         <v>15</v>
       </c>
@@ -1465,10 +1468,10 @@
       <c r="J15" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="17"/>
-    </row>
-    <row r="16" spans="1:11" ht="137" thickBot="1">
-      <c r="A16" s="15" t="s">
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16" spans="1:13" ht="171" thickBot="1">
+      <c r="A16" s="19" t="s">
         <v>39</v>
       </c>
       <c r="B16" s="8" t="s">
@@ -1496,8 +1499,8 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="35" thickBot="1">
-      <c r="A17" s="17"/>
+    <row r="17" spans="1:11" ht="52" thickBot="1">
+      <c r="A17" s="20"/>
       <c r="B17" s="7" t="s">
         <v>15</v>
       </c>
@@ -1522,7 +1525,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="409.6" thickBot="1">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="19" t="s">
         <v>43</v>
       </c>
       <c r="B18" s="8" t="s">
@@ -1546,12 +1549,12 @@
       <c r="J18" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="15" t="s">
+      <c r="K18" s="19" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="35" thickBot="1">
-      <c r="A19" s="17"/>
+      <c r="A19" s="20"/>
       <c r="B19" s="7" t="s">
         <v>15</v>
       </c>
@@ -1571,9 +1574,9 @@
       <c r="J19" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K19" s="17"/>
-    </row>
-    <row r="20" spans="1:11" ht="35" thickBot="1">
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20" spans="1:11" ht="52" thickBot="1">
       <c r="A20" s="8" t="s">
         <v>46</v>
       </c>
@@ -1603,7 +1606,7 @@
       </c>
     </row>
     <row r="21" spans="1:11" ht="35" thickBot="1">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="15" t="s">
         <v>51</v>
       </c>
       <c r="B21" s="7" t="s">
@@ -1625,12 +1628,12 @@
       <c r="J21" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="18" t="s">
+      <c r="K21" s="15" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="35" thickBot="1">
-      <c r="A22" s="19"/>
+      <c r="A22" s="16"/>
       <c r="B22" s="8" t="s">
         <v>15</v>
       </c>
@@ -1650,10 +1653,10 @@
       <c r="J22" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K22" s="19"/>
+      <c r="K22" s="16"/>
     </row>
     <row r="23" spans="1:11" ht="46" customHeight="1" thickBot="1">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B23" s="7" t="s">
@@ -1677,12 +1680,12 @@
       <c r="J23" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K23" s="18" t="s">
+      <c r="K23" s="15" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="18" thickBot="1">
-      <c r="A24" s="19"/>
+      <c r="A24" s="16"/>
       <c r="B24" s="8" t="s">
         <v>15</v>
       </c>
@@ -1704,10 +1707,10 @@
       <c r="J24" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K24" s="19"/>
+      <c r="K24" s="16"/>
     </row>
     <row r="25" spans="1:11" ht="18" thickBot="1">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="15" t="s">
         <v>55</v>
       </c>
       <c r="B25" s="7" t="s">
@@ -1731,12 +1734,12 @@
       <c r="J25" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K25" s="18" t="s">
+      <c r="K25" s="15" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="18" thickBot="1">
-      <c r="A26" s="19"/>
+      <c r="A26" s="16"/>
       <c r="B26" s="8" t="s">
         <v>15</v>
       </c>
@@ -1758,10 +1761,10 @@
       <c r="J26" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K26" s="19"/>
+      <c r="K26" s="16"/>
     </row>
     <row r="27" spans="1:11" ht="35" thickBot="1">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="15" t="s">
         <v>57</v>
       </c>
       <c r="B27" s="7" t="s">
@@ -1790,7 +1793,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="35" thickBot="1">
-      <c r="A28" s="19"/>
+      <c r="A28" s="16"/>
       <c r="B28" s="8" t="s">
         <v>15</v>
       </c>
@@ -1817,7 +1820,7 @@
       </c>
     </row>
     <row r="29" spans="1:11" ht="18" thickBot="1">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="15" t="s">
         <v>60</v>
       </c>
       <c r="B29" s="7" t="s">
@@ -1841,12 +1844,12 @@
       <c r="J29" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K29" s="18" t="s">
+      <c r="K29" s="15" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="18" thickBot="1">
-      <c r="A30" s="19"/>
+      <c r="A30" s="16"/>
       <c r="B30" s="8" t="s">
         <v>15</v>
       </c>
@@ -1868,31 +1871,31 @@
       <c r="J30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K30" s="19"/>
+      <c r="K30" s="16"/>
     </row>
     <row r="31" spans="1:11" ht="34">
-      <c r="A31" s="18" t="s">
+      <c r="A31" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
       <c r="E31" s="11"/>
-      <c r="F31" s="18">
+      <c r="F31" s="15">
         <v>25</v>
       </c>
-      <c r="G31" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="H31" s="18" t="s">
+      <c r="G31" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H31" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="I31" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="J31" s="18" t="s">
+      <c r="I31" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="J31" s="15" t="s">
         <v>12</v>
       </c>
       <c r="K31" s="11" t="s">
@@ -1900,22 +1903,22 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="35" thickBot="1">
-      <c r="A32" s="20"/>
-      <c r="B32" s="19"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="16"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="12"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
       <c r="K32" s="13" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="35" thickBot="1">
-      <c r="A33" s="19"/>
+      <c r="A33" s="16"/>
       <c r="B33" s="8" t="s">
         <v>15</v>
       </c>
@@ -1942,7 +1945,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="35" thickBot="1">
-      <c r="A34" s="18" t="s">
+      <c r="A34" s="15" t="s">
         <v>66</v>
       </c>
       <c r="B34" s="7" t="s">
@@ -1966,12 +1969,12 @@
       <c r="J34" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K34" s="18" t="s">
+      <c r="K34" s="15" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="35" thickBot="1">
-      <c r="A35" s="19"/>
+      <c r="A35" s="16"/>
       <c r="B35" s="8" t="s">
         <v>15</v>
       </c>
@@ -1993,10 +1996,10 @@
       <c r="J35" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K35" s="19"/>
+      <c r="K35" s="16"/>
     </row>
     <row r="36" spans="1:11" ht="35" thickBot="1">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="15" t="s">
         <v>69</v>
       </c>
       <c r="B36" s="7" t="s">
@@ -2020,12 +2023,12 @@
       <c r="J36" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K36" s="18" t="s">
+      <c r="K36" s="15" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="35" thickBot="1">
-      <c r="A37" s="19"/>
+      <c r="A37" s="16"/>
       <c r="B37" s="8" t="s">
         <v>15</v>
       </c>
@@ -2047,191 +2050,191 @@
       <c r="J37" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K37" s="19"/>
+      <c r="K37" s="16"/>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="18" t="s">
+      <c r="A38" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
-      <c r="F38" s="18">
+      <c r="F38" s="15">
         <v>30</v>
       </c>
-      <c r="G38" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="H38" s="18" t="s">
+      <c r="G38" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H38" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="I38" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="J38" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="K38" s="18" t="s">
+      <c r="I38" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="K38" s="15" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="17" thickBot="1">
-      <c r="A39" s="20"/>
-      <c r="B39" s="19"/>
+      <c r="A39" s="23"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
       <c r="E39" s="12"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
-      <c r="K39" s="20"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="25"/>
+      <c r="J39" s="25"/>
+      <c r="K39" s="23"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="20"/>
-      <c r="B40" s="15" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="19" t="s">
         <v>15</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
-      <c r="F40" s="15">
+      <c r="F40" s="19">
         <v>24</v>
       </c>
-      <c r="G40" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="H40" s="15" t="s">
+      <c r="G40" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="H40" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="I40" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="J40" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="K40" s="20"/>
+      <c r="I40" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="J40" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="K40" s="23"/>
     </row>
     <row r="41" spans="1:11" ht="17" thickBot="1">
-      <c r="A41" s="19"/>
-      <c r="B41" s="17"/>
+      <c r="A41" s="16"/>
+      <c r="B41" s="20"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="24"/>
-      <c r="J41" s="24"/>
-      <c r="K41" s="19"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="16"/>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
       <c r="E42" s="11"/>
-      <c r="F42" s="18">
+      <c r="F42" s="15">
         <v>18</v>
       </c>
-      <c r="G42" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="H42" s="18" t="s">
+      <c r="G42" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H42" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="I42" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="J42" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="K42" s="18" t="s">
+      <c r="I42" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="J42" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="K42" s="15" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="17" thickBot="1">
-      <c r="A43" s="20"/>
-      <c r="B43" s="19"/>
+      <c r="A43" s="23"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
       <c r="E43" s="12"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
-      <c r="K43" s="20"/>
+      <c r="F43" s="16"/>
+      <c r="G43" s="16"/>
+      <c r="H43" s="16"/>
+      <c r="I43" s="25"/>
+      <c r="J43" s="25"/>
+      <c r="K43" s="23"/>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="20"/>
-      <c r="B44" s="15" t="s">
+      <c r="A44" s="23"/>
+      <c r="B44" s="19" t="s">
         <v>15</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
-      <c r="F44" s="15">
+      <c r="F44" s="19">
         <v>18</v>
       </c>
-      <c r="G44" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="H44" s="15" t="s">
+      <c r="G44" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="H44" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="I44" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="J44" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="K44" s="20"/>
+      <c r="I44" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="J44" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="K44" s="23"/>
     </row>
     <row r="45" spans="1:11" ht="17" thickBot="1">
-      <c r="A45" s="19"/>
-      <c r="B45" s="17"/>
+      <c r="A45" s="16"/>
+      <c r="B45" s="20"/>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="24"/>
-      <c r="J45" s="24"/>
-      <c r="K45" s="19"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="20"/>
+      <c r="I45" s="22"/>
+      <c r="J45" s="22"/>
+      <c r="K45" s="16"/>
     </row>
     <row r="46" spans="1:11" ht="68">
-      <c r="A46" s="18" t="s">
+      <c r="A46" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="18" t="s">
+      <c r="B46" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C46" s="11"/>
       <c r="D46" s="11"/>
       <c r="E46" s="11"/>
-      <c r="F46" s="18">
+      <c r="F46" s="15">
         <v>25</v>
       </c>
-      <c r="G46" s="18" t="s">
+      <c r="G46" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="H46" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="I46" s="18" t="s">
+      <c r="H46" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="I46" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="J46" s="21" t="s">
+      <c r="J46" s="24" t="s">
         <v>22</v>
       </c>
       <c r="K46" s="11" t="s">
@@ -2239,39 +2242,39 @@
       </c>
     </row>
     <row r="47" spans="1:11" ht="17" thickBot="1">
-      <c r="A47" s="20"/>
-      <c r="B47" s="19"/>
+      <c r="A47" s="23"/>
+      <c r="B47" s="16"/>
       <c r="C47" s="12"/>
       <c r="D47" s="12"/>
       <c r="E47" s="12"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="19"/>
-      <c r="J47" s="22"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="25"/>
       <c r="K47" s="13"/>
     </row>
     <row r="48" spans="1:11" ht="68">
-      <c r="A48" s="20"/>
-      <c r="B48" s="15" t="s">
+      <c r="A48" s="23"/>
+      <c r="B48" s="19" t="s">
         <v>15</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
-      <c r="F48" s="15">
+      <c r="F48" s="19">
         <v>21</v>
       </c>
-      <c r="G48" s="15" t="s">
+      <c r="G48" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="H48" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="I48" s="15" t="s">
+      <c r="H48" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="I48" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="J48" s="23" t="s">
+      <c r="J48" s="21" t="s">
         <v>22</v>
       </c>
       <c r="K48" s="13" t="s">
@@ -2279,121 +2282,121 @@
       </c>
     </row>
     <row r="49" spans="1:11" ht="17" thickBot="1">
-      <c r="A49" s="19"/>
-      <c r="B49" s="17"/>
+      <c r="A49" s="16"/>
+      <c r="B49" s="20"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="24"/>
+      <c r="F49" s="20"/>
+      <c r="G49" s="20"/>
+      <c r="H49" s="20"/>
+      <c r="I49" s="20"/>
+      <c r="J49" s="22"/>
       <c r="K49" s="14"/>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="18" t="s">
+      <c r="A50" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C50" s="11"/>
       <c r="D50" s="11"/>
       <c r="E50" s="11"/>
-      <c r="F50" s="18">
+      <c r="F50" s="15">
         <v>25</v>
       </c>
-      <c r="G50" s="18" t="s">
+      <c r="G50" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="H50" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="I50" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="J50" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="K50" s="18" t="s">
+      <c r="H50" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="I50" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="J50" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="K50" s="15" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="17" thickBot="1">
-      <c r="A51" s="20"/>
-      <c r="B51" s="19"/>
+      <c r="A51" s="23"/>
+      <c r="B51" s="16"/>
       <c r="C51" s="12"/>
       <c r="D51" s="12"/>
       <c r="E51" s="12"/>
-      <c r="F51" s="19"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="19"/>
-      <c r="I51" s="22"/>
-      <c r="J51" s="22"/>
-      <c r="K51" s="20"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="25"/>
+      <c r="J51" s="25"/>
+      <c r="K51" s="23"/>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="20"/>
-      <c r="B52" s="15" t="s">
+      <c r="A52" s="23"/>
+      <c r="B52" s="19" t="s">
         <v>15</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
-      <c r="F52" s="15">
+      <c r="F52" s="19">
         <v>21</v>
       </c>
-      <c r="G52" s="15" t="s">
+      <c r="G52" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="H52" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="I52" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="J52" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="K52" s="20"/>
+      <c r="H52" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="I52" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="J52" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="K52" s="23"/>
     </row>
     <row r="53" spans="1:11" ht="17" thickBot="1">
-      <c r="A53" s="19"/>
-      <c r="B53" s="17"/>
+      <c r="A53" s="16"/>
+      <c r="B53" s="20"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="24"/>
-      <c r="J53" s="24"/>
-      <c r="K53" s="19"/>
+      <c r="F53" s="20"/>
+      <c r="G53" s="20"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="16"/>
     </row>
     <row r="54" spans="1:11" ht="68">
-      <c r="A54" s="18" t="s">
+      <c r="A54" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B54" s="18" t="s">
+      <c r="B54" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
-      <c r="F54" s="18">
+      <c r="F54" s="15">
         <v>18</v>
       </c>
-      <c r="G54" s="18" t="s">
+      <c r="G54" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="H54" s="18" t="s">
+      <c r="H54" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="I54" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="J54" s="18" t="s">
+      <c r="I54" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="J54" s="15" t="s">
         <v>12</v>
       </c>
       <c r="K54" s="11" t="s">
@@ -2401,20 +2404,20 @@
       </c>
     </row>
     <row r="55" spans="1:11" ht="17" thickBot="1">
-      <c r="A55" s="20"/>
-      <c r="B55" s="19"/>
+      <c r="A55" s="23"/>
+      <c r="B55" s="16"/>
       <c r="C55" s="12"/>
       <c r="D55" s="12"/>
       <c r="E55" s="12"/>
-      <c r="F55" s="19"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="19"/>
-      <c r="I55" s="19"/>
-      <c r="J55" s="19"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
+      <c r="J55" s="16"/>
       <c r="K55" s="13"/>
     </row>
     <row r="56" spans="1:11" ht="69" thickBot="1">
-      <c r="A56" s="19"/>
+      <c r="A56" s="16"/>
       <c r="B56" s="8" t="s">
         <v>15</v>
       </c>
@@ -2441,7 +2444,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="18" thickBot="1">
-      <c r="A57" s="18" t="s">
+      <c r="A57" s="15" t="s">
         <v>87</v>
       </c>
       <c r="B57" s="7" t="s">
@@ -2465,12 +2468,12 @@
       <c r="J57" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K57" s="18" t="s">
+      <c r="K57" s="15" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="18" thickBot="1">
-      <c r="A58" s="19"/>
+      <c r="A58" s="16"/>
       <c r="B58" s="8" t="s">
         <v>15</v>
       </c>
@@ -2492,10 +2495,10 @@
       <c r="J58" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K58" s="19"/>
+      <c r="K58" s="16"/>
     </row>
     <row r="59" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="15" t="s">
         <v>89</v>
       </c>
       <c r="B59" s="7" t="s">
@@ -2519,12 +2522,12 @@
       <c r="J59" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K59" s="18" t="s">
+      <c r="K59" s="15" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="18" thickBot="1">
-      <c r="A60" s="19"/>
+      <c r="A60" s="16"/>
       <c r="B60" s="8" t="s">
         <v>15</v>
       </c>
@@ -2546,10 +2549,10 @@
       <c r="J60" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K60" s="19"/>
+      <c r="K60" s="16"/>
     </row>
     <row r="61" spans="1:11" ht="52" thickBot="1">
-      <c r="A61" s="18" t="s">
+      <c r="A61" s="15" t="s">
         <v>91</v>
       </c>
       <c r="B61" s="7" t="s">
@@ -2578,7 +2581,7 @@
       </c>
     </row>
     <row r="62" spans="1:11" ht="52" thickBot="1">
-      <c r="A62" s="19"/>
+      <c r="A62" s="16"/>
       <c r="B62" s="8" t="s">
         <v>15</v>
       </c>
@@ -2605,7 +2608,7 @@
       </c>
     </row>
     <row r="63" spans="1:11" ht="52" thickBot="1">
-      <c r="A63" s="18" t="s">
+      <c r="A63" s="15" t="s">
         <v>95</v>
       </c>
       <c r="B63" s="7" t="s">
@@ -2634,7 +2637,7 @@
       </c>
     </row>
     <row r="64" spans="1:11" ht="52" thickBot="1">
-      <c r="A64" s="19"/>
+      <c r="A64" s="16"/>
       <c r="B64" s="8" t="s">
         <v>15</v>
       </c>
@@ -2661,7 +2664,7 @@
       </c>
     </row>
     <row r="65" spans="1:11" ht="35" thickBot="1">
-      <c r="A65" s="18" t="s">
+      <c r="A65" s="15" t="s">
         <v>98</v>
       </c>
       <c r="B65" s="7" t="s">
@@ -2685,12 +2688,12 @@
       <c r="J65" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K65" s="18" t="s">
+      <c r="K65" s="15" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="35" thickBot="1">
-      <c r="A66" s="19"/>
+      <c r="A66" s="16"/>
       <c r="B66" s="8" t="s">
         <v>15</v>
       </c>
@@ -2712,7 +2715,7 @@
       <c r="J66" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K66" s="19"/>
+      <c r="K66" s="16"/>
     </row>
     <row r="67" spans="1:11" ht="52" thickBot="1">
       <c r="A67" s="7" t="s">
@@ -2744,7 +2747,7 @@
       </c>
     </row>
     <row r="68" spans="1:11" ht="18" thickBot="1">
-      <c r="A68" s="15" t="s">
+      <c r="A68" s="19" t="s">
         <v>103</v>
       </c>
       <c r="B68" s="8" t="s">
@@ -2768,12 +2771,12 @@
       <c r="J68" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K68" s="15" t="s">
+      <c r="K68" s="19" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="18" thickBot="1">
-      <c r="A69" s="17"/>
+      <c r="A69" s="20"/>
       <c r="B69" s="7" t="s">
         <v>34</v>
       </c>
@@ -2795,10 +2798,10 @@
       <c r="J69" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K69" s="17"/>
-    </row>
-    <row r="70" spans="1:11" ht="52" thickBot="1">
-      <c r="A70" s="15" t="s">
+      <c r="K69" s="20"/>
+    </row>
+    <row r="70" spans="1:11" ht="69" thickBot="1">
+      <c r="A70" s="19" t="s">
         <v>106</v>
       </c>
       <c r="B70" s="8" t="s">
@@ -2826,8 +2829,8 @@
         <v>108</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="52" thickBot="1">
-      <c r="A71" s="17"/>
+    <row r="71" spans="1:11" ht="69" thickBot="1">
+      <c r="A71" s="20"/>
       <c r="B71" s="7" t="s">
         <v>15</v>
       </c>
@@ -2854,16 +2857,16 @@
       </c>
     </row>
     <row r="72" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A72" s="15" t="s">
+      <c r="A72" s="19" t="s">
         <v>110</v>
       </c>
       <c r="B72" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C72" s="25">
+      <c r="C72" s="17">
         <v>0</v>
       </c>
-      <c r="D72" s="25" t="s">
+      <c r="D72" s="17" t="s">
         <v>167</v>
       </c>
       <c r="E72" s="8"/>
@@ -2882,17 +2885,17 @@
       <c r="J72" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K72" s="15" t="s">
+      <c r="K72" s="19" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="18" thickBot="1">
-      <c r="A73" s="17"/>
+      <c r="A73" s="20"/>
       <c r="B73" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C73" s="26"/>
-      <c r="D73" s="26"/>
+      <c r="C73" s="18"/>
+      <c r="D73" s="18"/>
       <c r="E73" s="7"/>
       <c r="F73" s="7">
         <v>21</v>
@@ -2909,10 +2912,10 @@
       <c r="J73" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K73" s="17"/>
+      <c r="K73" s="20"/>
     </row>
     <row r="74" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A74" s="15" t="s">
+      <c r="A74" s="19" t="s">
         <v>112</v>
       </c>
       <c r="B74" s="8" t="s">
@@ -2936,12 +2939,12 @@
       <c r="J74" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K74" s="15" t="s">
+      <c r="K74" s="19" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="18" thickBot="1">
-      <c r="A75" s="17"/>
+      <c r="A75" s="20"/>
       <c r="B75" s="7" t="s">
         <v>15</v>
       </c>
@@ -2963,10 +2966,10 @@
       <c r="J75" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K75" s="17"/>
+      <c r="K75" s="20"/>
     </row>
     <row r="76" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A76" s="15" t="s">
+      <c r="A76" s="19" t="s">
         <v>114</v>
       </c>
       <c r="B76" s="8" t="s">
@@ -2990,12 +2993,12 @@
       <c r="J76" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K76" s="15" t="s">
+      <c r="K76" s="19" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="18" thickBot="1">
-      <c r="A77" s="17"/>
+      <c r="A77" s="20"/>
       <c r="B77" s="7" t="s">
         <v>34</v>
       </c>
@@ -3017,10 +3020,10 @@
       <c r="J77" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K77" s="17"/>
+      <c r="K77" s="20"/>
     </row>
     <row r="78" spans="1:11" ht="52" thickBot="1">
-      <c r="A78" s="15" t="s">
+      <c r="A78" s="19" t="s">
         <v>116</v>
       </c>
       <c r="B78" s="8" t="s">
@@ -3049,7 +3052,7 @@
       </c>
     </row>
     <row r="79" spans="1:11" ht="52" thickBot="1">
-      <c r="A79" s="17"/>
+      <c r="A79" s="20"/>
       <c r="B79" s="7" t="s">
         <v>15</v>
       </c>
@@ -3076,7 +3079,7 @@
       </c>
     </row>
     <row r="80" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A80" s="15" t="s">
+      <c r="A80" s="19" t="s">
         <v>119</v>
       </c>
       <c r="B80" s="8" t="s">
@@ -3100,12 +3103,12 @@
       <c r="J80" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K80" s="15" t="s">
+      <c r="K80" s="19" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="18" thickBot="1">
-      <c r="A81" s="17"/>
+      <c r="A81" s="20"/>
       <c r="B81" s="7" t="s">
         <v>15</v>
       </c>
@@ -3127,10 +3130,10 @@
       <c r="J81" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K81" s="17"/>
+      <c r="K81" s="20"/>
     </row>
     <row r="82" spans="1:11" ht="94" customHeight="1" thickBot="1">
-      <c r="A82" s="15" t="s">
+      <c r="A82" s="19" t="s">
         <v>121</v>
       </c>
       <c r="B82" s="8" t="s">
@@ -3154,12 +3157,12 @@
       <c r="J82" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K82" s="15" t="s">
+      <c r="K82" s="19" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="18" thickBot="1">
-      <c r="A83" s="17"/>
+      <c r="A83" s="20"/>
       <c r="B83" s="7" t="s">
         <v>15</v>
       </c>
@@ -3181,10 +3184,10 @@
       <c r="J83" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K83" s="17"/>
+      <c r="K83" s="20"/>
     </row>
     <row r="84" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A84" s="15" t="s">
+      <c r="A84" s="19" t="s">
         <v>123</v>
       </c>
       <c r="B84" s="8" t="s">
@@ -3208,12 +3211,12 @@
       <c r="J84" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K84" s="15" t="s">
+      <c r="K84" s="19" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="18" thickBot="1">
-      <c r="A85" s="17"/>
+      <c r="A85" s="20"/>
       <c r="B85" s="7" t="s">
         <v>15</v>
       </c>
@@ -3235,10 +3238,10 @@
       <c r="J85" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K85" s="17"/>
+      <c r="K85" s="20"/>
     </row>
     <row r="86" spans="1:11" ht="35" thickBot="1">
-      <c r="A86" s="15" t="s">
+      <c r="A86" s="19" t="s">
         <v>125</v>
       </c>
       <c r="B86" s="8" t="s">
@@ -3262,12 +3265,12 @@
       <c r="J86" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K86" s="15" t="s">
+      <c r="K86" s="19" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="35" thickBot="1">
-      <c r="A87" s="17"/>
+      <c r="A87" s="20"/>
       <c r="B87" s="7" t="s">
         <v>15</v>
       </c>
@@ -3289,10 +3292,10 @@
       <c r="J87" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K87" s="17"/>
+      <c r="K87" s="20"/>
     </row>
     <row r="88" spans="1:11" ht="35" thickBot="1">
-      <c r="A88" s="15" t="s">
+      <c r="A88" s="19" t="s">
         <v>127</v>
       </c>
       <c r="B88" s="8" t="s">
@@ -3316,12 +3319,12 @@
       <c r="J88" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K88" s="15" t="s">
+      <c r="K88" s="19" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="35" thickBot="1">
-      <c r="A89" s="17"/>
+      <c r="A89" s="20"/>
       <c r="B89" s="7" t="s">
         <v>15</v>
       </c>
@@ -3343,10 +3346,10 @@
       <c r="J89" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K89" s="17"/>
-    </row>
-    <row r="90" spans="1:11" ht="35" thickBot="1">
-      <c r="A90" s="15" t="s">
+      <c r="K89" s="20"/>
+    </row>
+    <row r="90" spans="1:11" ht="52" thickBot="1">
+      <c r="A90" s="19" t="s">
         <v>129</v>
       </c>
       <c r="B90" s="8" t="s">
@@ -3375,7 +3378,7 @@
       </c>
     </row>
     <row r="91" spans="1:11" ht="103" thickBot="1">
-      <c r="A91" s="17"/>
+      <c r="A91" s="20"/>
       <c r="B91" s="7" t="s">
         <v>15</v>
       </c>
@@ -3402,7 +3405,7 @@
       </c>
     </row>
     <row r="92" spans="1:11" ht="18" thickBot="1">
-      <c r="A92" s="15" t="s">
+      <c r="A92" s="19" t="s">
         <v>133</v>
       </c>
       <c r="B92" s="8" t="s">
@@ -3426,12 +3429,12 @@
       <c r="J92" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K92" s="15" t="s">
+      <c r="K92" s="19" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="18" thickBot="1">
-      <c r="A93" s="17"/>
+      <c r="A93" s="20"/>
       <c r="B93" s="7" t="s">
         <v>15</v>
       </c>
@@ -3453,10 +3456,10 @@
       <c r="J93" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K93" s="17"/>
+      <c r="K93" s="20"/>
     </row>
     <row r="94" spans="1:11" ht="18" thickBot="1">
-      <c r="A94" s="15" t="s">
+      <c r="A94" s="19" t="s">
         <v>135</v>
       </c>
       <c r="B94" s="8" t="s">
@@ -3480,12 +3483,12 @@
       <c r="J94" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K94" s="15" t="s">
+      <c r="K94" s="19" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="18" thickBot="1">
-      <c r="A95" s="17"/>
+      <c r="A95" s="20"/>
       <c r="B95" s="7" t="s">
         <v>15</v>
       </c>
@@ -3507,10 +3510,10 @@
       <c r="J95" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K95" s="17"/>
+      <c r="K95" s="20"/>
     </row>
     <row r="96" spans="1:11" ht="35" thickBot="1">
-      <c r="A96" s="15" t="s">
+      <c r="A96" s="19" t="s">
         <v>137</v>
       </c>
       <c r="B96" s="8" t="s">
@@ -3534,12 +3537,12 @@
       <c r="J96" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K96" s="15" t="s">
+      <c r="K96" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="35" thickBot="1">
-      <c r="A97" s="17"/>
+      <c r="A97" s="20"/>
       <c r="B97" s="7" t="s">
         <v>15</v>
       </c>
@@ -3561,10 +3564,10 @@
       <c r="J97" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K97" s="17"/>
+      <c r="K97" s="20"/>
     </row>
     <row r="98" spans="1:11" ht="52" thickBot="1">
-      <c r="A98" s="15" t="s">
+      <c r="A98" s="19" t="s">
         <v>139</v>
       </c>
       <c r="B98" s="8" t="s">
@@ -3593,7 +3596,7 @@
       </c>
     </row>
     <row r="99" spans="1:11" ht="52" thickBot="1">
-      <c r="A99" s="17"/>
+      <c r="A99" s="20"/>
       <c r="B99" s="7" t="s">
         <v>15</v>
       </c>
@@ -3620,7 +3623,7 @@
       </c>
     </row>
     <row r="100" spans="1:11" ht="52" thickBot="1">
-      <c r="A100" s="15" t="s">
+      <c r="A100" s="19" t="s">
         <v>144</v>
       </c>
       <c r="B100" s="8" t="s">
@@ -3649,7 +3652,7 @@
       </c>
     </row>
     <row r="101" spans="1:11" ht="52" thickBot="1">
-      <c r="A101" s="17"/>
+      <c r="A101" s="20"/>
       <c r="B101" s="7" t="s">
         <v>15</v>
       </c>
@@ -3676,7 +3679,7 @@
       </c>
     </row>
     <row r="102" spans="1:11" ht="18" thickBot="1">
-      <c r="A102" s="15" t="s">
+      <c r="A102" s="19" t="s">
         <v>147</v>
       </c>
       <c r="B102" s="8" t="s">
@@ -3700,12 +3703,12 @@
       <c r="J102" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K102" s="15" t="s">
+      <c r="K102" s="19" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="18" thickBot="1">
-      <c r="A103" s="17"/>
+      <c r="A103" s="20"/>
       <c r="B103" s="7" t="s">
         <v>15</v>
       </c>
@@ -3727,10 +3730,10 @@
       <c r="J103" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K103" s="17"/>
+      <c r="K103" s="20"/>
     </row>
     <row r="104" spans="1:11" ht="52" thickBot="1">
-      <c r="A104" s="15" t="s">
+      <c r="A104" s="19" t="s">
         <v>149</v>
       </c>
       <c r="B104" s="8" t="s">
@@ -3759,7 +3762,7 @@
       </c>
     </row>
     <row r="105" spans="1:11" ht="52" thickBot="1">
-      <c r="A105" s="17"/>
+      <c r="A105" s="20"/>
       <c r="B105" s="7" t="s">
         <v>15</v>
       </c>
@@ -3786,28 +3789,28 @@
       </c>
     </row>
     <row r="106" spans="1:11" ht="34">
-      <c r="A106" s="15" t="s">
+      <c r="A106" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="B106" s="15" t="s">
+      <c r="B106" s="19" t="s">
         <v>8</v>
       </c>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
-      <c r="F106" s="15">
+      <c r="F106" s="19">
         <v>21</v>
       </c>
-      <c r="G106" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="H106" s="15" t="s">
+      <c r="G106" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="H106" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="I106" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="J106" s="23" t="s">
+      <c r="I106" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="J106" s="21" t="s">
         <v>22</v>
       </c>
       <c r="K106" s="3" t="s">
@@ -3815,22 +3818,22 @@
       </c>
     </row>
     <row r="107" spans="1:11" ht="35" thickBot="1">
-      <c r="A107" s="17"/>
-      <c r="B107" s="17"/>
+      <c r="A107" s="20"/>
+      <c r="B107" s="20"/>
       <c r="C107" s="4"/>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
-      <c r="F107" s="17"/>
-      <c r="G107" s="24"/>
-      <c r="H107" s="17"/>
-      <c r="I107" s="17"/>
-      <c r="J107" s="24"/>
+      <c r="F107" s="20"/>
+      <c r="G107" s="22"/>
+      <c r="H107" s="20"/>
+      <c r="I107" s="20"/>
+      <c r="J107" s="22"/>
       <c r="K107" s="4" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A108" s="18" t="s">
+      <c r="A108" s="15" t="s">
         <v>156</v>
       </c>
       <c r="B108" s="7" t="s">
@@ -3854,12 +3857,12 @@
       <c r="J108" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K108" s="18" t="s">
+      <c r="K108" s="15" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="18" thickBot="1">
-      <c r="A109" s="19"/>
+      <c r="A109" s="16"/>
       <c r="B109" s="8" t="s">
         <v>15</v>
       </c>
@@ -3881,10 +3884,10 @@
       <c r="J109" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K109" s="19"/>
+      <c r="K109" s="16"/>
     </row>
     <row r="110" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A110" s="18" t="s">
+      <c r="A110" s="15" t="s">
         <v>158</v>
       </c>
       <c r="B110" s="7" t="s">
@@ -3908,12 +3911,12 @@
       <c r="J110" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K110" s="18" t="s">
+      <c r="K110" s="15" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="18" thickBot="1">
-      <c r="A111" s="19"/>
+      <c r="A111" s="16"/>
       <c r="B111" s="8" t="s">
         <v>15</v>
       </c>
@@ -3935,10 +3938,10 @@
       <c r="J111" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K111" s="19"/>
+      <c r="K111" s="16"/>
     </row>
     <row r="112" spans="1:11" ht="30" customHeight="1" thickBot="1">
-      <c r="A112" s="18" t="s">
+      <c r="A112" s="15" t="s">
         <v>160</v>
       </c>
       <c r="B112" s="7" t="s">
@@ -3962,12 +3965,12 @@
       <c r="J112" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K112" s="18" t="s">
+      <c r="K112" s="15" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="18" thickBot="1">
-      <c r="A113" s="19"/>
+      <c r="A113" s="16"/>
       <c r="B113" s="8" t="s">
         <v>15</v>
       </c>
@@ -3989,10 +3992,10 @@
       <c r="J113" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K113" s="19"/>
+      <c r="K113" s="16"/>
     </row>
     <row r="114" spans="1:11" ht="18" thickBot="1">
-      <c r="A114" s="18" t="s">
+      <c r="A114" s="15" t="s">
         <v>162</v>
       </c>
       <c r="B114" s="7" t="s">
@@ -4016,12 +4019,12 @@
       <c r="J114" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K114" s="18" t="s">
+      <c r="K114" s="15" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="18" thickBot="1">
-      <c r="A115" s="19"/>
+      <c r="A115" s="16"/>
       <c r="B115" s="8" t="s">
         <v>15</v>
       </c>
@@ -4043,10 +4046,10 @@
       <c r="J115" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K115" s="19"/>
+      <c r="K115" s="16"/>
     </row>
     <row r="116" spans="1:11" ht="35" thickBot="1">
-      <c r="A116" s="18" t="s">
+      <c r="A116" s="15" t="s">
         <v>164</v>
       </c>
       <c r="B116" s="7" t="s">
@@ -4070,12 +4073,12 @@
       <c r="J116" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K116" s="18" t="s">
+      <c r="K116" s="15" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="35" thickBot="1">
-      <c r="A117" s="19"/>
+      <c r="A117" s="16"/>
       <c r="B117" s="8" t="s">
         <v>15</v>
       </c>
@@ -4097,13 +4100,148 @@
       <c r="J117" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K117" s="19"/>
+      <c r="K117" s="16"/>
     </row>
     <row r="118" spans="1:11">
       <c r="A118" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="159">
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="K21:K22"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="K34:K35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="K36:K37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="K38:K41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="H40:H41"/>
+    <mergeCell ref="I40:I41"/>
+    <mergeCell ref="J40:J41"/>
+    <mergeCell ref="J42:J43"/>
+    <mergeCell ref="K42:K45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="H44:H45"/>
+    <mergeCell ref="I44:I45"/>
+    <mergeCell ref="J44:J45"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="H42:H43"/>
+    <mergeCell ref="I42:I43"/>
+    <mergeCell ref="J46:J47"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="H48:H49"/>
+    <mergeCell ref="I48:I49"/>
+    <mergeCell ref="J48:J49"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:G47"/>
+    <mergeCell ref="H46:H47"/>
+    <mergeCell ref="I46:I47"/>
+    <mergeCell ref="J50:J51"/>
+    <mergeCell ref="K50:K53"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="H52:H53"/>
+    <mergeCell ref="I52:I53"/>
+    <mergeCell ref="J52:J53"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="G50:G51"/>
+    <mergeCell ref="H50:H51"/>
+    <mergeCell ref="I50:I51"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="K65:K66"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="K68:K69"/>
+    <mergeCell ref="A70:A71"/>
+    <mergeCell ref="J54:J55"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="K57:K58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="K59:K60"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="G54:G55"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="I54:I55"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="A80:A81"/>
+    <mergeCell ref="K80:K81"/>
+    <mergeCell ref="A82:A83"/>
+    <mergeCell ref="K82:K83"/>
+    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="K84:K85"/>
+    <mergeCell ref="A72:A73"/>
+    <mergeCell ref="K72:K73"/>
+    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="K74:K75"/>
+    <mergeCell ref="A76:A77"/>
+    <mergeCell ref="K76:K77"/>
+    <mergeCell ref="A96:A97"/>
+    <mergeCell ref="K96:K97"/>
+    <mergeCell ref="A98:A99"/>
+    <mergeCell ref="A100:A101"/>
+    <mergeCell ref="A86:A87"/>
+    <mergeCell ref="K86:K87"/>
+    <mergeCell ref="A88:A89"/>
+    <mergeCell ref="K88:K89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="A92:A93"/>
+    <mergeCell ref="K92:K93"/>
     <mergeCell ref="A114:A115"/>
     <mergeCell ref="K114:K115"/>
     <mergeCell ref="A116:A117"/>
@@ -4128,141 +4266,6 @@
     <mergeCell ref="J106:J107"/>
     <mergeCell ref="A94:A95"/>
     <mergeCell ref="K94:K95"/>
-    <mergeCell ref="A96:A97"/>
-    <mergeCell ref="K96:K97"/>
-    <mergeCell ref="A98:A99"/>
-    <mergeCell ref="A100:A101"/>
-    <mergeCell ref="A86:A87"/>
-    <mergeCell ref="K86:K87"/>
-    <mergeCell ref="A88:A89"/>
-    <mergeCell ref="K88:K89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="A92:A93"/>
-    <mergeCell ref="K92:K93"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="A80:A81"/>
-    <mergeCell ref="K80:K81"/>
-    <mergeCell ref="A82:A83"/>
-    <mergeCell ref="K82:K83"/>
-    <mergeCell ref="A84:A85"/>
-    <mergeCell ref="K84:K85"/>
-    <mergeCell ref="A72:A73"/>
-    <mergeCell ref="K72:K73"/>
-    <mergeCell ref="A74:A75"/>
-    <mergeCell ref="K74:K75"/>
-    <mergeCell ref="A76:A77"/>
-    <mergeCell ref="K76:K77"/>
-    <mergeCell ref="A63:A64"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="K65:K66"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="K68:K69"/>
-    <mergeCell ref="A70:A71"/>
-    <mergeCell ref="J54:J55"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="K57:K58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="K59:K60"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="G54:G55"/>
-    <mergeCell ref="H54:H55"/>
-    <mergeCell ref="I54:I55"/>
-    <mergeCell ref="J50:J51"/>
-    <mergeCell ref="K50:K53"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="H52:H53"/>
-    <mergeCell ref="I52:I53"/>
-    <mergeCell ref="J52:J53"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="G50:G51"/>
-    <mergeCell ref="H50:H51"/>
-    <mergeCell ref="I50:I51"/>
-    <mergeCell ref="J46:J47"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="G48:G49"/>
-    <mergeCell ref="H48:H49"/>
-    <mergeCell ref="I48:I49"/>
-    <mergeCell ref="J48:J49"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="H46:H47"/>
-    <mergeCell ref="I46:I47"/>
-    <mergeCell ref="J42:J43"/>
-    <mergeCell ref="K42:K45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="F44:F45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="H44:H45"/>
-    <mergeCell ref="I44:I45"/>
-    <mergeCell ref="J44:J45"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="H42:H43"/>
-    <mergeCell ref="I42:I43"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="K38:K41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="G40:G41"/>
-    <mergeCell ref="H40:H41"/>
-    <mergeCell ref="I40:I41"/>
-    <mergeCell ref="J40:J41"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="K34:K35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="K36:K37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="F38:F39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="K29:K30"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>